<commit_message>
Corregir excel_exporter: faltaban lineas para guardar el archivo
</commit_message>
<xml_diff>
--- a/data/salida_cortes.xlsx
+++ b/data/salida_cortes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,12 +459,22 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Duración (h)</t>
+          <t>Duracion (h)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
           <t>CP&gt;2</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Fuente Distrito</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Archivo</t>
         </is>
       </c>
     </row>
@@ -499,10 +509,14 @@
           <t>Ica</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Ica</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Asociación De Vivienda San Luis Gonzaga De Ica, Habilitación Urbana Chacarilla, Urb. Chacarilla S/N, Urbanización Casuarinas – Etapas (I, II, III, IV, V, VI), Las Casuarinas (Techo Propio), Urbanización El Haras – Etapas (I, II, III, IV, V, VI), C.P. Cachiche – Parque, Á.V. Ricardo Palma (I y II) – Cachiche,</t>
+          <t>Asociación De Vivienda San Luis Gonzaga De Ica, Habilitación Urbana Chacarilla, Urb. Chacarilla S/N, Urbanización Casuarinas – Etapas (I, II, III, IV, V, VI), Las Casuarinas (Techo Propio), Urbanización El Haras – Etapas (I, II, III, IV, V, VI), C.P. Cachiche – Parque, A.V. Ricardo Palma (I y II) – Cachiche,</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -511,6 +525,16 @@
       <c r="J2" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Ubigeo (coincidencia en referencia)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>imagen_1.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>